<commit_message>
Treat IMO import as class text
</commit_message>
<xml_diff>
--- a/public/templates/imo-oog-modelo.xlsx
+++ b/public/templates/imo-oog-modelo.xlsx
@@ -421,7 +421,7 @@
         <v>CSLU1234567</v>
       </c>
       <c r="C2" t="str">
-        <v>Sim</v>
+        <v>IMO CLASS 3 UN 1203</v>
       </c>
       <c r="D2" t="str">
         <v>Nao</v>
@@ -435,7 +435,7 @@
         <v>TEMU7654321</v>
       </c>
       <c r="C3" t="str">
-        <v>Nao</v>
+        <v/>
       </c>
       <c r="D3" t="str">
         <v>Sim</v>

</xml_diff>